<commit_message>
WIP checkpoint: Parts 2/3 chapter edits in progress (Ch 18, 22-26, 34), not yet checked
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V4hHp37cV1PSzEtykqYjK1
</commit_message>
<xml_diff>
--- a/Data Science/Analyst-to-Architect/companion/ch18/reports/riverstone_2025-12.xlsx
+++ b/Data Science/Analyst-to-Architect/companion/ch18/reports/riverstone_2025-12.xlsx
@@ -16,27 +16,39 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+  <si>
+    <t>measure</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>Net revenue (₹)</t>
+  </si>
+  <si>
+    <t>Orders</t>
+  </si>
+  <si>
+    <t>Customers</t>
+  </si>
+  <si>
+    <t>Average order value (₹)</t>
+  </si>
+  <si>
+    <t>Gross margin (%)</t>
+  </si>
+  <si>
+    <t>Share of target (%)</t>
+  </si>
+  <si>
+    <t>segment</t>
+  </si>
   <si>
     <t>net_revenue</t>
   </si>
   <si>
     <t>orders</t>
-  </si>
-  <si>
-    <t>customers</t>
-  </si>
-  <si>
-    <t>average_order_value</t>
-  </si>
-  <si>
-    <t>gross_margin_pct</t>
-  </si>
-  <si>
-    <t>pct_of_target</t>
-  </si>
-  <si>
-    <t>segment</t>
   </si>
   <si>
     <t>Retail</t>
@@ -405,46 +417,65 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="2" width="26.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="B2">
+        <v>87266803.75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="B3">
+        <v>4047</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="B4">
+        <v>3240</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2">
-        <v>87266803.75</v>
-      </c>
-      <c r="B2">
-        <v>4047</v>
-      </c>
-      <c r="C2">
-        <v>3240</v>
-      </c>
-      <c r="D2">
+      <c r="B5">
         <v>21563.33</v>
       </c>
-      <c r="E2">
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
         <v>27.6</v>
       </c>
-      <c r="F2">
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7">
         <v>94.40000000000001</v>
       </c>
     </row>
@@ -455,54 +486,54 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
-    <col min="2" max="4" width="16.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B2" s="1">
         <v>42213835</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2">
         <v>2106</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B3" s="1">
         <v>23584620</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3">
         <v>855</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B4" s="1">
         <v>21468348.75</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4">
         <v>1086</v>
       </c>
     </row>
@@ -513,24 +544,24 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
-    <col min="2" max="4" width="16.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B2" s="1">
         <v>18622125</v>
@@ -538,7 +569,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B3" s="1">
         <v>16770845</v>
@@ -546,7 +577,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B4" s="1">
         <v>15806606.5</v>
@@ -554,7 +585,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B5" s="1">
         <v>11903220</v>
@@ -562,7 +593,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B6" s="1">
         <v>10850176</v>
@@ -570,7 +601,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B7" s="1">
         <v>10138020</v>
@@ -578,7 +609,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B8" s="1">
         <v>3175811.25</v>

</xml_diff>